<commit_message>
Add shipper weight to total weight calculations
</commit_message>
<xml_diff>
--- a/shippers.xlsx
+++ b/shippers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://elcompanies-my.sharepoint.com/personal/ahaider1_estee_com1/Documents/Desktop/shippers/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://elcompanies-my.sharepoint.com/personal/ahaider1_estee_com1/Documents/Desktop/PACKAGING TOOL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{56BFFBE9-8ACB-45F2-85D8-161E94F5F106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B258BEFD-8E4D-45C7-A7B9-70BF670C49FC}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{56BFFBE9-8ACB-45F2-85D8-161E94F5F106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00A2CE74-224D-49E7-BD46-4BD22B606CCC}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-1965" windowWidth="29040" windowHeight="15720" xr2:uid="{C43C274C-2242-4FEC-875B-B7D5CA08FB3C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C43C274C-2242-4FEC-875B-B7D5CA08FB3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>E6-SHIPPER</t>
   </si>
@@ -108,6 +108,33 @@
   </si>
   <si>
     <t>SRMX-01-0901 (of SRMX-01-0902 Y-label)</t>
+  </si>
+  <si>
+    <t>WEIGHT</t>
+  </si>
+  <si>
+    <t>0,22 KG</t>
+  </si>
+  <si>
+    <t>0,42 KG</t>
+  </si>
+  <si>
+    <t>0,46 KG</t>
+  </si>
+  <si>
+    <t>0,50 KG</t>
+  </si>
+  <si>
+    <t>0.22 KG</t>
+  </si>
+  <si>
+    <t>0.38 KG</t>
+  </si>
+  <si>
+    <t>0,32 KG</t>
+  </si>
+  <si>
+    <t>0,35 KG</t>
   </si>
 </sst>
 </file>
@@ -178,18 +205,18 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,345 +554,342 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="34.54296875" customWidth="1"/>
-    <col min="3" max="4" width="10.453125" customWidth="1"/>
-    <col min="5" max="5" width="14.08984375" customWidth="1"/>
-    <col min="6" max="7" width="16.08984375" customWidth="1"/>
-    <col min="8" max="8" width="8.6328125" customWidth="1"/>
+    <col min="1" max="2" width="34.5703125" customWidth="1"/>
+    <col min="3" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" customWidth="1"/>
+    <col min="6" max="7" width="16.140625" customWidth="1"/>
+    <col min="8" max="8" width="8.5703125" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="12" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.90625" customWidth="1"/>
-    <col min="14" max="14" width="23.453125" customWidth="1"/>
+    <col min="10" max="12" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" customWidth="1"/>
+    <col min="14" max="14" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="7" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+      <c r="G1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="5">
         <v>382</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="5">
         <v>282</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="5">
         <v>137</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="5">
         <f t="shared" ref="F2:F9" si="0">E2*D2*C2</f>
         <v>14758188</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="4"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="N2" s="3"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="5">
         <v>382</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="5">
         <v>282</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="5">
         <v>173</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="5">
         <f t="shared" si="0"/>
         <v>18636252</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="4"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
+      <c r="N3" s="3"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="5">
         <v>382</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="5">
         <v>282</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="5">
         <v>229</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="5">
         <f t="shared" si="0"/>
         <v>24668796</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>28</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="4"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="N4" s="3"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="5">
         <v>273</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="5">
         <v>229</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="5">
         <v>110</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="5">
         <f t="shared" si="0"/>
         <v>6876870</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="4"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="5">
         <v>245</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="5">
         <v>220</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="5">
         <v>125</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="5">
         <f t="shared" si="0"/>
         <v>6737500</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="4"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+      <c r="N6" s="3"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="5">
         <v>298</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="5">
         <v>246</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="5">
         <v>152</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="5">
         <f t="shared" si="0"/>
         <v>11142816</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="4"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
+      <c r="N7" s="3"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="5">
         <v>405</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="5">
         <v>265</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="5">
         <v>104</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="5">
         <f t="shared" si="0"/>
         <v>11161800</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="4"/>
-    </row>
-    <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="N8" s="3"/>
+    </row>
+    <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="5">
         <v>350</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="5">
         <v>273</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="5">
         <v>106</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="5">
         <f t="shared" si="0"/>
         <v>10128300</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="4"/>
-    </row>
-    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8" t="s">
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="5">
         <v>265</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="5">
         <v>226</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="5">
         <v>164</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="5">
         <f t="shared" ref="F10" si="1">E10*D10*C10</f>
         <v>9821960</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="4"/>
-    </row>
-    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="N10" s="3"/>
+    </row>
+    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="8"/>
       <c r="I11" s="1"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="4"/>
-    </row>
-    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+      <c r="N11" s="3"/>
+    </row>
+    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5">
         <f t="shared" ref="F12" si="2">E12*D12*C12</f>
         <v>0</v>
       </c>
+      <c r="G12" s="8"/>
       <c r="I12" s="1"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="4"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
+      <c r="N12" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Restore report and data files from previous commit
</commit_message>
<xml_diff>
--- a/shippers.xlsx
+++ b/shippers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://elcompanies-my.sharepoint.com/personal/ahaider1_estee_com1/Documents/Desktop/PACKAGING TOOL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://elcompanies-my.sharepoint.com/personal/ahaider1_estee_com1/Documents/Desktop/shippers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{56BFFBE9-8ACB-45F2-85D8-161E94F5F106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00A2CE74-224D-49E7-BD46-4BD22B606CCC}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{56BFFBE9-8ACB-45F2-85D8-161E94F5F106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B258BEFD-8E4D-45C7-A7B9-70BF670C49FC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C43C274C-2242-4FEC-875B-B7D5CA08FB3C}"/>
+    <workbookView xWindow="-57720" yWindow="-1965" windowWidth="29040" windowHeight="15720" xr2:uid="{C43C274C-2242-4FEC-875B-B7D5CA08FB3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>E6-SHIPPER</t>
   </si>
@@ -108,33 +108,6 @@
   </si>
   <si>
     <t>SRMX-01-0901 (of SRMX-01-0902 Y-label)</t>
-  </si>
-  <si>
-    <t>WEIGHT</t>
-  </si>
-  <si>
-    <t>0,22 KG</t>
-  </si>
-  <si>
-    <t>0,42 KG</t>
-  </si>
-  <si>
-    <t>0,46 KG</t>
-  </si>
-  <si>
-    <t>0,50 KG</t>
-  </si>
-  <si>
-    <t>0.22 KG</t>
-  </si>
-  <si>
-    <t>0.38 KG</t>
-  </si>
-  <si>
-    <t>0,32 KG</t>
-  </si>
-  <si>
-    <t>0,35 KG</t>
   </si>
 </sst>
 </file>
@@ -205,18 +178,18 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,342 +527,345 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="34.5703125" customWidth="1"/>
-    <col min="3" max="4" width="10.42578125" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" customWidth="1"/>
-    <col min="6" max="7" width="16.140625" customWidth="1"/>
-    <col min="8" max="8" width="8.5703125" customWidth="1"/>
+    <col min="1" max="2" width="34.54296875" customWidth="1"/>
+    <col min="3" max="4" width="10.453125" customWidth="1"/>
+    <col min="5" max="5" width="14.08984375" customWidth="1"/>
+    <col min="6" max="7" width="16.08984375" customWidth="1"/>
+    <col min="8" max="8" width="8.6328125" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="12" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.85546875" customWidth="1"/>
-    <col min="14" max="14" width="23.42578125" customWidth="1"/>
+    <col min="10" max="12" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.90625" customWidth="1"/>
+    <col min="14" max="14" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="7">
         <v>382</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="7">
         <v>282</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="7">
         <v>137</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="7">
         <f t="shared" ref="F2:F9" si="0">E2*D2*C2</f>
         <v>14758188</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>26</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="N2" s="3"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="M2" s="3"/>
+      <c r="N2" s="4"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="7">
         <v>382</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="7">
         <v>282</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="7">
         <v>173</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="7">
         <f t="shared" si="0"/>
         <v>18636252</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>27</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
-      <c r="N3" s="3"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="M3" s="3"/>
+      <c r="N3" s="4"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="7">
         <v>382</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="7">
         <v>282</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="7">
         <v>229</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="7">
         <f t="shared" si="0"/>
         <v>24668796</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>28</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
-      <c r="N4" s="3"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="M4" s="3"/>
+      <c r="N4" s="4"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="7">
         <v>273</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="7">
         <v>229</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="7">
         <v>110</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="7">
         <f t="shared" si="0"/>
         <v>6876870</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>29</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
-      <c r="N5" s="3"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="M5" s="3"/>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="7">
         <v>245</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="7">
         <v>220</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="7">
         <v>125</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="7">
         <f t="shared" si="0"/>
         <v>6737500</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>30</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-      <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="M6" s="3"/>
+      <c r="N6" s="4"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="7">
         <v>298</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="7">
         <v>246</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="7">
         <v>152</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="7">
         <f t="shared" si="0"/>
         <v>11142816</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>32</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
-      <c r="N7" s="3"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="M7" s="3"/>
+      <c r="N7" s="4"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="7">
         <v>405</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="7">
         <v>265</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="7">
         <v>104</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="7">
         <f t="shared" si="0"/>
         <v>11161800</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>31</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
-      <c r="N8" s="3"/>
-    </row>
-    <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="M8" s="3"/>
+      <c r="N8" s="4"/>
+    </row>
+    <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="7">
         <v>350</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="7">
         <v>273</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="7">
         <v>106</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="7">
         <f t="shared" si="0"/>
         <v>10128300</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>32</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="M9" s="3"/>
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="7">
         <v>265</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="7">
         <v>226</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="7">
         <v>164</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="7">
         <f t="shared" ref="F10" si="1">E10*D10*C10</f>
         <v>9821960</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
-      <c r="N10" s="3"/>
-    </row>
-    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="8"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="4"/>
+    </row>
+    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
       <c r="I11" s="1"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
-      <c r="N11" s="3"/>
-    </row>
-    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="M11" s="3"/>
+      <c r="N11" s="4"/>
+    </row>
+    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7">
         <f t="shared" ref="F12" si="2">E12*D12*C12</f>
         <v>0</v>
       </c>
-      <c r="G12" s="8"/>
       <c r="I12" s="1"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="N12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="4"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>